<commit_message>
change: returned Morris_Noise to collored plots
</commit_message>
<xml_diff>
--- a/notebooks/Phase_methods_analytics/Global_analytics/Morris/morris_mu_highlighted.xlsx
+++ b/notebooks/Phase_methods_analytics/Global_analytics/Morris/morris_mu_highlighted.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,40 +474,292 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
+          <t>MP</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>7.63e-3</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>-2.76</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>-0.14</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>6.89e-3</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>-0.56</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>-0.77</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>ZCRR</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.22e-3</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>-0.15</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>-1.82</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4.91e-3</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>-0.06</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>FFT</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>-4.6e-4</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>-0.19</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>-0.22</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-8.01e-4</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-6.08e-3</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-9.74e-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>HB</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-1.95e-3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>-9.8e-4</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>-0.02</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-0.02</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>5.86e-4</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>-0.08</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>-0.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>XCOR</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>0.48</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>-0.65</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>-0.17</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>-2.19e-4</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>-0.05</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>-0.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>-1.09e-4</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0.47</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>-0.52</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>-0.3</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>-6.24e-4</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>-4.64e-3</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2.67e-3</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>0.06</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>-0.13</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>0.11</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2.61e-4</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>4.07e-3</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>SWFR</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2.12e-4</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1.11e-3</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>-0.02</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>-1.69e-3</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>-0.03</t>
         </is>

</xml_diff>